<commit_message>
[FIX] sale: test int-id assumptions (sales team members, import template dates)
- test_sale_order TestSalesTeam.setUpClass wrote member_ids = [4, user.id], a raw
  int user id 4 mixed with a uuid; use Command.set with base.user_admin + user_in_team.
- quotations_import_template.xlsx used =NOW()/=TODAY() formula cells for Order Date /
  Expiration. base_import reads xlsx with data_only=True, which returns the cached
  formula value (None here) -> date_order imported as NULL -> not-null violation. Use
  literal datetime values so the required date_order is populated. (Surfaced only after
  the earlier "Deco Addict"->"Acme Corporation" partner-name fix let the import proceed.)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Vu4e83fYXhR4oircH5GXnb
</commit_message>
<xml_diff>
--- a/addons/sale/static/xls/quotations_import_template.xlsx
+++ b/addons/sale/static/xls/quotations_import_template.xlsx
@@ -16,8 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mm/yy"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd hh:mm:ss"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -83,7 +85,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -128,6 +130,12 @@
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -405,13 +413,11 @@
           <t>Azure Interior</t>
         </is>
       </c>
-      <c r="C2" s="14">
-        <f>NOW()</f>
-        <v/>
-      </c>
-      <c r="D2" s="14">
-        <f>TODAY()+30</f>
-        <v/>
+      <c r="C2" s="16" t="n">
+        <v>45292</v>
+      </c>
+      <c r="D2" s="17" t="n">
+        <v>45322</v>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
@@ -470,13 +476,11 @@
           <t>Azure Interior, Brandon Freeman</t>
         </is>
       </c>
-      <c r="C4" s="14">
-        <f>TODAY()</f>
-        <v/>
-      </c>
-      <c r="D4" s="14">
-        <f>TODAY()+60</f>
-        <v/>
+      <c r="C4" s="16" t="n">
+        <v>45292</v>
+      </c>
+      <c r="D4" s="17" t="n">
+        <v>45352</v>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
@@ -535,13 +539,11 @@
           <t>Acme Corporation</t>
         </is>
       </c>
-      <c r="C6" s="14">
-        <f>TODAY()</f>
-        <v/>
-      </c>
-      <c r="D6" s="14">
-        <f>TODAY()+90</f>
-        <v/>
+      <c r="C6" s="16" t="n">
+        <v>45292</v>
+      </c>
+      <c r="D6" s="17" t="n">
+        <v>45382</v>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>

</xml_diff>